<commit_message>
history data is all right.
</commit_message>
<xml_diff>
--- a/Others/Quant模型设计.xlsx
+++ b/Others/Quant模型设计.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9180"/>
+    <workbookView windowWidth="15960" windowHeight="8652" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="T00" sheetId="1" r:id="rId1"/>
@@ -3085,7 +3085,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14994890" y="10421620"/>
+          <a:off x="14914880" y="10421620"/>
           <a:ext cx="1118870" cy="2019300"/>
         </a:xfrm>
         <a:prstGeom prst="rightBrace">
@@ -3377,7 +3377,7 @@
     <col min="2" max="2" width="9" style="3"/>
     <col min="3" max="3" width="12.1111111111111" style="3" customWidth="1"/>
     <col min="4" max="4" width="12.1759259259259" customWidth="1"/>
-    <col min="5" max="5" width="48.0185185185185" customWidth="1"/>
+    <col min="5" max="5" width="46.8518518518519" customWidth="1"/>
     <col min="6" max="6" width="35.4444444444444" customWidth="1"/>
     <col min="7" max="7" width="31.8888888888889" customWidth="1"/>
     <col min="8" max="8" width="43.6666666666667" customWidth="1"/>

</xml_diff>